<commit_message>
Week 18 B2b WM
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 18/White_Mulberry/other_channels.xlsx
+++ b/data/raw/sales/Week 18/White_Mulberry/other_channels.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Week 17\Week 18\raw\sales\Week 18\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 18\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C90F74-4FE3-47A7-891F-DCD9E71689CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F05BFD-EC32-4A69-9ABF-7D3EB27ED9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1p Sales" sheetId="9" r:id="rId1"/>
     <sheet name="BI Worldwide" sheetId="10" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="11" r:id="rId3"/>
+    <sheet name="B2B" sheetId="11" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1p Sales'!$C$1:$F$67</definedName>
@@ -191,26 +191,31 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">

</xml_diff>